<commit_message>
fix: correct premium data, gender labels, plan names, and add premi table section
- Replace placeholder premium data with correct values from PDFs
- Change gender labels from Pria/Wanita to Laki-Laki/Perempuan
- Update plan names to include coverage amounts (e.g. Plan 1 (100/200))
- Update data validation dropdowns for gender and plan
- Change subtitles to KALKULATOR PREMI/KONTRIBUSI format
- Add TABEL LENGKAP PREMI section showing all plans
- Add copyright footer

Co-authored-by: petrusjakub <76829088+petrusjakub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalkulator_Premi_MiUHC.xlsx
+++ b/Kalkulator_Premi_MiUHC.xlsx
@@ -9,12 +9,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>PETRUS JAKUB MANULIFE 087781896087</t>
   </si>
   <si>
-    <t>MiUHC Konvensional - Efektif 1 September 2025</t>
+    <t>KALKULATOR PREMI MIUHC - Berlaku mulai 1 September 2025</t>
   </si>
   <si>
     <t>Nama Tertanggung:</t>
@@ -26,7 +26,7 @@
     <t>Jenis Kelamin:</t>
   </si>
   <si>
-    <t>Pria</t>
+    <t>Laki-Laki</t>
   </si>
   <si>
     <t>Tanggal Lahir:</t>
@@ -38,7 +38,7 @@
     <t>Plan:</t>
   </si>
   <si>
-    <t>Plan 1</t>
+    <t>Plan 1 (100/200)</t>
   </si>
   <si>
     <t>HASIL PERHITUNGAN</t>
@@ -53,49 +53,79 @@
     <t>Key</t>
   </si>
   <si>
-    <t>Plan 2</t>
-  </si>
-  <si>
-    <t>Plan 3</t>
-  </si>
-  <si>
-    <t>Plan 4</t>
-  </si>
-  <si>
-    <t>Plan 5</t>
-  </si>
-  <si>
-    <t>Pria_20-30</t>
-  </si>
-  <si>
-    <t>Pria_31-40</t>
-  </si>
-  <si>
-    <t>Pria_41-50</t>
-  </si>
-  <si>
-    <t>Pria_51-60</t>
-  </si>
-  <si>
-    <t>Pria_61-70</t>
-  </si>
-  <si>
-    <t>Wanita_20-30</t>
-  </si>
-  <si>
-    <t>Wanita_31-40</t>
-  </si>
-  <si>
-    <t>Wanita_41-50</t>
-  </si>
-  <si>
-    <t>Wanita_51-60</t>
-  </si>
-  <si>
-    <t>Wanita_61-70</t>
-  </si>
-  <si>
-    <t>MiUHC Syariah - Efektif 1 Januari 2024</t>
+    <t>Plan 2 (200/400)</t>
+  </si>
+  <si>
+    <t>Plan 3 (400/800)</t>
+  </si>
+  <si>
+    <t>Plan 4 (600/1.200)</t>
+  </si>
+  <si>
+    <t>Plan 5 (1.000/2.000)</t>
+  </si>
+  <si>
+    <t>Laki-Laki_20-30</t>
+  </si>
+  <si>
+    <t>Laki-Laki_31-40</t>
+  </si>
+  <si>
+    <t>Laki-Laki_41-50</t>
+  </si>
+  <si>
+    <t>Laki-Laki_51-60</t>
+  </si>
+  <si>
+    <t>Laki-Laki_61-70</t>
+  </si>
+  <si>
+    <t>Perempuan_20-30</t>
+  </si>
+  <si>
+    <t>Perempuan_31-40</t>
+  </si>
+  <si>
+    <t>Perempuan_41-50</t>
+  </si>
+  <si>
+    <t>Perempuan_51-60</t>
+  </si>
+  <si>
+    <t>Perempuan_61-70</t>
+  </si>
+  <si>
+    <t>TABEL LENGKAP PREMI MIUHC</t>
+  </si>
+  <si>
+    <t>Usia</t>
+  </si>
+  <si>
+    <t>Perempuan</t>
+  </si>
+  <si>
+    <t>20-30</t>
+  </si>
+  <si>
+    <t>31-40</t>
+  </si>
+  <si>
+    <t>41-50</t>
+  </si>
+  <si>
+    <t>51-60</t>
+  </si>
+  <si>
+    <t>61-70</t>
+  </si>
+  <si>
+    <t>© PETRUS JAKUB MANULIFE 087781896087</t>
+  </si>
+  <si>
+    <t>KALKULATOR KONTRIBUSI MIUHC SYARIAH - Berlaku mulai 1 Januari 2024</t>
+  </si>
+  <si>
+    <t>TABEL LENGKAP KONTRIBUSI MIUHC SYARIAH</t>
   </si>
 </sst>
 </file>
@@ -298,19 +328,19 @@
         <v>18</v>
       </c>
       <c r="B16" s="5">
-        <v>3500000</v>
+        <v>2380000</v>
       </c>
       <c r="C16" s="5">
-        <v>5200000</v>
+        <v>3570000</v>
       </c>
       <c r="D16" s="5">
-        <v>7800000</v>
+        <v>5950000</v>
       </c>
       <c r="E16" s="5">
-        <v>11500000</v>
+        <v>8330000</v>
       </c>
       <c r="F16" s="5">
-        <v>16800000</v>
+        <v>11900000</v>
       </c>
     </row>
     <row r="17">
@@ -318,19 +348,19 @@
         <v>19</v>
       </c>
       <c r="B17" s="5">
-        <v>4200000</v>
+        <v>3710000</v>
       </c>
       <c r="C17" s="5">
-        <v>6300000</v>
+        <v>5570000</v>
       </c>
       <c r="D17" s="5">
-        <v>9500000</v>
+        <v>9280000</v>
       </c>
       <c r="E17" s="5">
-        <v>14000000</v>
+        <v>12990000</v>
       </c>
       <c r="F17" s="5">
-        <v>20500000</v>
+        <v>18560000</v>
       </c>
     </row>
     <row r="18">
@@ -338,19 +368,19 @@
         <v>20</v>
       </c>
       <c r="B18" s="5">
-        <v>5800000</v>
+        <v>5040000</v>
       </c>
       <c r="C18" s="5">
-        <v>8700000</v>
+        <v>7560000</v>
       </c>
       <c r="D18" s="5">
-        <v>13000000</v>
+        <v>12600000</v>
       </c>
       <c r="E18" s="5">
-        <v>19500000</v>
+        <v>17640000</v>
       </c>
       <c r="F18" s="5">
-        <v>28500000</v>
+        <v>25200000</v>
       </c>
     </row>
     <row r="19">
@@ -358,19 +388,19 @@
         <v>21</v>
       </c>
       <c r="B19" s="5">
-        <v>8500000</v>
+        <v>6370000</v>
       </c>
       <c r="C19" s="5">
-        <v>12500000</v>
+        <v>9560000</v>
       </c>
       <c r="D19" s="5">
-        <v>18800000</v>
+        <v>15930000</v>
       </c>
       <c r="E19" s="5">
-        <v>28000000</v>
+        <v>22300000</v>
       </c>
       <c r="F19" s="5">
-        <v>41000000</v>
+        <v>31860000</v>
       </c>
     </row>
     <row r="20">
@@ -378,19 +408,19 @@
         <v>22</v>
       </c>
       <c r="B20" s="5">
-        <v>12000000</v>
+        <v>8360000</v>
       </c>
       <c r="C20" s="5">
-        <v>17500000</v>
+        <v>12540000</v>
       </c>
       <c r="D20" s="5">
-        <v>26000000</v>
+        <v>20900000</v>
       </c>
       <c r="E20" s="5">
-        <v>39000000</v>
+        <v>29260000</v>
       </c>
       <c r="F20" s="5">
-        <v>57000000</v>
+        <v>41800000</v>
       </c>
     </row>
     <row r="21">
@@ -398,19 +428,19 @@
         <v>23</v>
       </c>
       <c r="B21" s="5">
-        <v>3800000</v>
+        <v>3430000</v>
       </c>
       <c r="C21" s="5">
-        <v>5600000</v>
+        <v>5150000</v>
       </c>
       <c r="D21" s="5">
-        <v>8400000</v>
+        <v>8580000</v>
       </c>
       <c r="E21" s="5">
-        <v>12500000</v>
+        <v>12010000</v>
       </c>
       <c r="F21" s="5">
-        <v>18200000</v>
+        <v>17160000</v>
       </c>
     </row>
     <row r="22">
@@ -418,19 +448,19 @@
         <v>24</v>
       </c>
       <c r="B22" s="5">
-        <v>4500000</v>
+        <v>4760000</v>
       </c>
       <c r="C22" s="5">
-        <v>6800000</v>
+        <v>7150000</v>
       </c>
       <c r="D22" s="5">
-        <v>10200000</v>
+        <v>11910000</v>
       </c>
       <c r="E22" s="5">
-        <v>15200000</v>
+        <v>16670000</v>
       </c>
       <c r="F22" s="5">
-        <v>22000000</v>
+        <v>23820000</v>
       </c>
     </row>
     <row r="23">
@@ -438,19 +468,19 @@
         <v>25</v>
       </c>
       <c r="B23" s="5">
-        <v>6200000</v>
+        <v>6090000</v>
       </c>
       <c r="C23" s="5">
-        <v>9300000</v>
+        <v>9140000</v>
       </c>
       <c r="D23" s="5">
-        <v>14000000</v>
+        <v>15230000</v>
       </c>
       <c r="E23" s="5">
-        <v>21000000</v>
+        <v>21320000</v>
       </c>
       <c r="F23" s="5">
-        <v>30500000</v>
+        <v>30460000</v>
       </c>
     </row>
     <row r="24">
@@ -458,19 +488,19 @@
         <v>26</v>
       </c>
       <c r="B24" s="5">
-        <v>9000000</v>
+        <v>7420000</v>
       </c>
       <c r="C24" s="5">
-        <v>13200000</v>
+        <v>11140000</v>
       </c>
       <c r="D24" s="5">
-        <v>20000000</v>
+        <v>18560000</v>
       </c>
       <c r="E24" s="5">
-        <v>30000000</v>
+        <v>25980000</v>
       </c>
       <c r="F24" s="5">
-        <v>43500000</v>
+        <v>37120000</v>
       </c>
     </row>
     <row r="25">
@@ -478,19 +508,391 @@
         <v>27</v>
       </c>
       <c r="B25" s="5">
-        <v>12800000</v>
+        <v>9410000</v>
       </c>
       <c r="C25" s="5">
-        <v>18500000</v>
+        <v>14120000</v>
       </c>
       <c r="D25" s="5">
-        <v>27500000</v>
+        <v>23530000</v>
       </c>
       <c r="E25" s="5">
-        <v>41500000</v>
+        <v>32940000</v>
       </c>
       <c r="F25" s="5">
-        <v>60000000</v>
+        <v>47060000</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" t="s" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B31" s="5">
+        <v>2380000</v>
+      </c>
+      <c r="C31" s="5">
+        <v>3430000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B32" s="5">
+        <v>3710000</v>
+      </c>
+      <c r="C32" s="5">
+        <v>4760000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B33" s="5">
+        <v>5040000</v>
+      </c>
+      <c r="C33" s="5">
+        <v>6090000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B34" s="5">
+        <v>6370000</v>
+      </c>
+      <c r="C34" s="5">
+        <v>7420000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B35" s="5">
+        <v>8360000</v>
+      </c>
+      <c r="C35" s="5">
+        <v>9410000</v>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B39" s="5">
+        <v>3570000</v>
+      </c>
+      <c r="C39" s="5">
+        <v>5150000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B40" s="5">
+        <v>5570000</v>
+      </c>
+      <c r="C40" s="5">
+        <v>7150000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B41" s="5">
+        <v>7560000</v>
+      </c>
+      <c r="C41" s="5">
+        <v>9140000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B42" s="5">
+        <v>9560000</v>
+      </c>
+      <c r="C42" s="5">
+        <v>11140000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B43" s="5">
+        <v>12540000</v>
+      </c>
+      <c r="C43" s="5">
+        <v>14120000</v>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B46" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C46" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B47" s="5">
+        <v>5950000</v>
+      </c>
+      <c r="C47" s="5">
+        <v>8580000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5">
+        <v>9280000</v>
+      </c>
+      <c r="C48" s="5">
+        <v>11910000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B49" s="5">
+        <v>12600000</v>
+      </c>
+      <c r="C49" s="5">
+        <v>15230000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B50" s="5">
+        <v>15930000</v>
+      </c>
+      <c r="C50" s="5">
+        <v>18560000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B51" s="5">
+        <v>20900000</v>
+      </c>
+      <c r="C51" s="5">
+        <v>23530000</v>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" t="s" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B54" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B55" s="5">
+        <v>8330000</v>
+      </c>
+      <c r="C55" s="5">
+        <v>12010000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B56" s="5">
+        <v>12990000</v>
+      </c>
+      <c r="C56" s="5">
+        <v>16670000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B57" s="5">
+        <v>17640000</v>
+      </c>
+      <c r="C57" s="5">
+        <v>21320000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B58" s="5">
+        <v>22300000</v>
+      </c>
+      <c r="C58" s="5">
+        <v>25980000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B59" s="5">
+        <v>29260000</v>
+      </c>
+      <c r="C59" s="5">
+        <v>32940000</v>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B62" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B63" s="5">
+        <v>11900000</v>
+      </c>
+      <c r="C63" s="5">
+        <v>17160000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B64" s="5">
+        <v>18560000</v>
+      </c>
+      <c r="C64" s="5">
+        <v>23820000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B65" s="5">
+        <v>25200000</v>
+      </c>
+      <c r="C65" s="5">
+        <v>30460000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B66" s="5">
+        <v>31860000</v>
+      </c>
+      <c r="C66" s="5">
+        <v>37120000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B67" s="5">
+        <v>41800000</v>
+      </c>
+      <c r="C67" s="5">
+        <v>47060000</v>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -499,10 +901,10 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B5">
-      <formula1>"Pria,Wanita"</formula1>
+      <formula1>"Laki-Laki,Perempuan"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B8">
-      <formula1>"Plan 1,Plan 2,Plan 3,Plan 4,Plan 5"</formula1>
+      <formula1>"Plan 1 (100/200),Plan 2 (200/400),Plan 3 (400/800),Plan 4 (600/1.200),Plan 5 (1.000/2.000)"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -526,7 +928,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="1">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3"/>
@@ -622,19 +1024,19 @@
         <v>18</v>
       </c>
       <c r="B16" s="5">
-        <v>3500000</v>
+        <v>2380000</v>
       </c>
       <c r="C16" s="5">
-        <v>5200000</v>
+        <v>3570000</v>
       </c>
       <c r="D16" s="5">
-        <v>7800000</v>
+        <v>5950000</v>
       </c>
       <c r="E16" s="5">
-        <v>11500000</v>
+        <v>8330000</v>
       </c>
       <c r="F16" s="5">
-        <v>16800000</v>
+        <v>11900000</v>
       </c>
     </row>
     <row r="17">
@@ -642,19 +1044,19 @@
         <v>19</v>
       </c>
       <c r="B17" s="5">
-        <v>4200000</v>
+        <v>3710000</v>
       </c>
       <c r="C17" s="5">
-        <v>6300000</v>
+        <v>5570000</v>
       </c>
       <c r="D17" s="5">
-        <v>9500000</v>
+        <v>9280000</v>
       </c>
       <c r="E17" s="5">
-        <v>14000000</v>
+        <v>12990000</v>
       </c>
       <c r="F17" s="5">
-        <v>20500000</v>
+        <v>18560000</v>
       </c>
     </row>
     <row r="18">
@@ -662,19 +1064,19 @@
         <v>20</v>
       </c>
       <c r="B18" s="5">
-        <v>5800000</v>
+        <v>5040000</v>
       </c>
       <c r="C18" s="5">
-        <v>8700000</v>
+        <v>7560000</v>
       </c>
       <c r="D18" s="5">
-        <v>13000000</v>
+        <v>12600000</v>
       </c>
       <c r="E18" s="5">
-        <v>19500000</v>
+        <v>17640000</v>
       </c>
       <c r="F18" s="5">
-        <v>28500000</v>
+        <v>25200000</v>
       </c>
     </row>
     <row r="19">
@@ -682,19 +1084,19 @@
         <v>21</v>
       </c>
       <c r="B19" s="5">
-        <v>8500000</v>
+        <v>6370000</v>
       </c>
       <c r="C19" s="5">
-        <v>12500000</v>
+        <v>9560000</v>
       </c>
       <c r="D19" s="5">
-        <v>18800000</v>
+        <v>15930000</v>
       </c>
       <c r="E19" s="5">
-        <v>28000000</v>
+        <v>22300000</v>
       </c>
       <c r="F19" s="5">
-        <v>41000000</v>
+        <v>31860000</v>
       </c>
     </row>
     <row r="20">
@@ -702,19 +1104,19 @@
         <v>22</v>
       </c>
       <c r="B20" s="5">
-        <v>12000000</v>
+        <v>8360000</v>
       </c>
       <c r="C20" s="5">
-        <v>17500000</v>
+        <v>12540000</v>
       </c>
       <c r="D20" s="5">
-        <v>26000000</v>
+        <v>20900000</v>
       </c>
       <c r="E20" s="5">
-        <v>39000000</v>
+        <v>29260000</v>
       </c>
       <c r="F20" s="5">
-        <v>57000000</v>
+        <v>41800000</v>
       </c>
     </row>
     <row r="21">
@@ -722,19 +1124,19 @@
         <v>23</v>
       </c>
       <c r="B21" s="5">
-        <v>3800000</v>
+        <v>3430000</v>
       </c>
       <c r="C21" s="5">
-        <v>5600000</v>
+        <v>5150000</v>
       </c>
       <c r="D21" s="5">
-        <v>8400000</v>
+        <v>8580000</v>
       </c>
       <c r="E21" s="5">
-        <v>12500000</v>
+        <v>12010000</v>
       </c>
       <c r="F21" s="5">
-        <v>18200000</v>
+        <v>17160000</v>
       </c>
     </row>
     <row r="22">
@@ -742,19 +1144,19 @@
         <v>24</v>
       </c>
       <c r="B22" s="5">
-        <v>4500000</v>
+        <v>4760000</v>
       </c>
       <c r="C22" s="5">
-        <v>6800000</v>
+        <v>7150000</v>
       </c>
       <c r="D22" s="5">
-        <v>10200000</v>
+        <v>11910000</v>
       </c>
       <c r="E22" s="5">
-        <v>15200000</v>
+        <v>16670000</v>
       </c>
       <c r="F22" s="5">
-        <v>22000000</v>
+        <v>23820000</v>
       </c>
     </row>
     <row r="23">
@@ -762,19 +1164,19 @@
         <v>25</v>
       </c>
       <c r="B23" s="5">
-        <v>6200000</v>
+        <v>6090000</v>
       </c>
       <c r="C23" s="5">
-        <v>9300000</v>
+        <v>9140000</v>
       </c>
       <c r="D23" s="5">
-        <v>14000000</v>
+        <v>15230000</v>
       </c>
       <c r="E23" s="5">
-        <v>21000000</v>
+        <v>21320000</v>
       </c>
       <c r="F23" s="5">
-        <v>30500000</v>
+        <v>30460000</v>
       </c>
     </row>
     <row r="24">
@@ -782,19 +1184,19 @@
         <v>26</v>
       </c>
       <c r="B24" s="5">
-        <v>9000000</v>
+        <v>7420000</v>
       </c>
       <c r="C24" s="5">
-        <v>13200000</v>
+        <v>11140000</v>
       </c>
       <c r="D24" s="5">
-        <v>20000000</v>
+        <v>18560000</v>
       </c>
       <c r="E24" s="5">
-        <v>30000000</v>
+        <v>25980000</v>
       </c>
       <c r="F24" s="5">
-        <v>43500000</v>
+        <v>37120000</v>
       </c>
     </row>
     <row r="25">
@@ -802,19 +1204,391 @@
         <v>27</v>
       </c>
       <c r="B25" s="5">
-        <v>12800000</v>
+        <v>9410000</v>
       </c>
       <c r="C25" s="5">
-        <v>18500000</v>
+        <v>14120000</v>
       </c>
       <c r="D25" s="5">
-        <v>27500000</v>
+        <v>23530000</v>
       </c>
       <c r="E25" s="5">
-        <v>41500000</v>
+        <v>32940000</v>
       </c>
       <c r="F25" s="5">
-        <v>60000000</v>
+        <v>47060000</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" t="s" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B31" s="5">
+        <v>2380000</v>
+      </c>
+      <c r="C31" s="5">
+        <v>3430000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B32" s="5">
+        <v>3710000</v>
+      </c>
+      <c r="C32" s="5">
+        <v>4760000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B33" s="5">
+        <v>5040000</v>
+      </c>
+      <c r="C33" s="5">
+        <v>6090000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B34" s="5">
+        <v>6370000</v>
+      </c>
+      <c r="C34" s="5">
+        <v>7420000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B35" s="5">
+        <v>8360000</v>
+      </c>
+      <c r="C35" s="5">
+        <v>9410000</v>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B39" s="5">
+        <v>3570000</v>
+      </c>
+      <c r="C39" s="5">
+        <v>5150000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B40" s="5">
+        <v>5570000</v>
+      </c>
+      <c r="C40" s="5">
+        <v>7150000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B41" s="5">
+        <v>7560000</v>
+      </c>
+      <c r="C41" s="5">
+        <v>9140000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B42" s="5">
+        <v>9560000</v>
+      </c>
+      <c r="C42" s="5">
+        <v>11140000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B43" s="5">
+        <v>12540000</v>
+      </c>
+      <c r="C43" s="5">
+        <v>14120000</v>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B46" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C46" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B47" s="5">
+        <v>5950000</v>
+      </c>
+      <c r="C47" s="5">
+        <v>8580000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5">
+        <v>9280000</v>
+      </c>
+      <c r="C48" s="5">
+        <v>11910000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B49" s="5">
+        <v>12600000</v>
+      </c>
+      <c r="C49" s="5">
+        <v>15230000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B50" s="5">
+        <v>15930000</v>
+      </c>
+      <c r="C50" s="5">
+        <v>18560000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B51" s="5">
+        <v>20900000</v>
+      </c>
+      <c r="C51" s="5">
+        <v>23530000</v>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" t="s" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B54" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B55" s="5">
+        <v>8330000</v>
+      </c>
+      <c r="C55" s="5">
+        <v>12010000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B56" s="5">
+        <v>12990000</v>
+      </c>
+      <c r="C56" s="5">
+        <v>16670000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B57" s="5">
+        <v>17640000</v>
+      </c>
+      <c r="C57" s="5">
+        <v>21320000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B58" s="5">
+        <v>22300000</v>
+      </c>
+      <c r="C58" s="5">
+        <v>25980000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B59" s="5">
+        <v>29260000</v>
+      </c>
+      <c r="C59" s="5">
+        <v>32940000</v>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="B62" t="s" s="1">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B63" s="5">
+        <v>11900000</v>
+      </c>
+      <c r="C63" s="5">
+        <v>17160000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B64" s="5">
+        <v>18560000</v>
+      </c>
+      <c r="C64" s="5">
+        <v>23820000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B65" s="5">
+        <v>25200000</v>
+      </c>
+      <c r="C65" s="5">
+        <v>30460000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B66" s="5">
+        <v>31860000</v>
+      </c>
+      <c r="C66" s="5">
+        <v>37120000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B67" s="5">
+        <v>41800000</v>
+      </c>
+      <c r="C67" s="5">
+        <v>47060000</v>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -823,10 +1597,10 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="B5">
-      <formula1>"Pria,Wanita"</formula1>
+      <formula1>"Laki-Laki,Perempuan"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B8">
-      <formula1>"Plan 1,Plan 2,Plan 3,Plan 4,Plan 5"</formula1>
+      <formula1>"Plan 1 (100/200),Plan 2 (200/400),Plan 3 (400/800),Plan 4 (600/1.200),Plan 5 (1.000/2.000)"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>